<commit_message>
Add CSC program database structure
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:28:29Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:28:29Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:36:57Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:36:57Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Add professor database queue and workbook
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:36:57Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:36:57Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:46:19Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:46:19Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Add professor snapshot and initial PKU faculty data
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:46:19Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:46:19Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:53:14Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:53:14Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Add C9 professor first-pass coverage
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:53:14Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:53:14Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:02:33Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:02:33Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Add richer professor detail fields
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:02:33Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:02:33Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:08:20Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:08:20Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Import local professor spreadsheets into database
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:08:20Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:08:20Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:17:48Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:17:48Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Expand professor details for C9 and top 985
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:17:48Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:17:48Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:30:42Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:30:42Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Add professor outreach and more imported rows
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:30:42Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:30:42Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:41:36Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:41:36Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>

<commit_message>
Track outreach metrics in professor report
</commit_message>
<xml_diff>
--- a/workbooks/china_university_tiers.xlsx
+++ b/workbooks/china_university_tiers.xlsx
@@ -27,8 +27,8 @@
   <dc:title>China University Tiers</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:41:36Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:41:36Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T05:57:17Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T05:57:17Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>